<commit_message>
feature: Change the homework script to start with 'result'=output business JSON, use 'data' for the host list and 'result' for each business result. Update the built-in inspection script, report template, and instructions together
</commit_message>
<xml_diff>
--- a/server/apps/workflow_orchestration/assets/templates/health-inspection-example.xlsx
+++ b/server/apps/workflow_orchestration/assets/templates/health-inspection-example.xlsx
@@ -724,7 +724,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status != 'SUCCESS' %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status != 'SUCCESS' %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -739,17 +739,17 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.critical_count }}</t>
+          <t>{{ r.result.critical_count }}</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.warning_count }}</t>
+          <t>{{ r.result.warning_count }}</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.normal_count }}</t>
+          <t>{{ r.result.normal_count }}</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
@@ -761,7 +761,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status == 'SUCCESS' and r.data.critical_count &gt; 0 %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status == 'SUCCESS' and r.result.critical_count &gt; 0 %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -776,17 +776,17 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.critical_count }}</t>
+          <t>{{ r.result.critical_count }}</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.warning_count }}</t>
+          <t>{{ r.result.warning_count }}</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.normal_count }}</t>
+          <t>{{ r.result.normal_count }}</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr">
@@ -798,7 +798,7 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status == 'SUCCESS' and r.data.critical_count == 0 and r.data.warning_count &gt; 0 %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status == 'SUCCESS' and r.result.critical_count == 0 and r.result.warning_count &gt; 0 %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -813,17 +813,17 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.critical_count }}</t>
+          <t>{{ r.result.critical_count }}</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.warning_count }}</t>
+          <t>{{ r.result.warning_count }}</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.normal_count }}</t>
+          <t>{{ r.result.normal_count }}</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
@@ -835,7 +835,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status == 'SUCCESS' and r.data.critical_count == 0 and r.data.warning_count == 0 %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status == 'SUCCESS' and r.result.critical_count == 0 and r.result.warning_count == 0 %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
@@ -850,17 +850,17 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.critical_count }}</t>
+          <t>{{ r.result.critical_count }}</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.warning_count }}</t>
+          <t>{{ r.result.warning_count }}</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>{{ r.data.normal_count }}</t>
+          <t>{{ r.result.normal_count }}</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -1046,7 +1046,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results %}{% for m in r.data.critical|default([]) %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data %}{% for m in r.result.critical|default([]) %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -1146,7 +1146,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results %}{% for m in r.data.warning|default([]) %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data %}{% for m in r.result.warning|default([]) %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -1264,7 +1264,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status != 'SUCCESS' %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status != 'SUCCESS' %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -1316,7 +1316,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status == 'SUCCESS' and r.data.critical_count &gt; 0 %}{% for m in r.data.metrics %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status == 'SUCCESS' and r.result.critical_count &gt; 0 %}{% for m in r.result.metrics %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status == 'SUCCESS' and r.data.critical_count == 0 and r.data.warning_count &gt; 0 %}{% for m in r.data.metrics %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status == 'SUCCESS' and r.result.critical_count == 0 and r.result.warning_count &gt; 0 %}{% for m in r.result.metrics %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -1420,7 +1420,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>{% tr %}{% for r in results if r.status == 'SUCCESS' and r.data.critical_count == 0 and r.data.warning_count == 0 %}{% for m in r.data.metrics %}{{ r.target.name }}</t>
+          <t>{% tr %}{% for r in data if r.status == 'SUCCESS' and r.result.critical_count == 0 and r.result.warning_count == 0 %}{% for m in r.result.metrics %}{{ r.target.name }}</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">

</xml_diff>